<commit_message>
Move HudIconPath column next to IconPath in items table
HudIconPath를 IconPath 바로 오른쪽으로 이동하고 컬럼 폭과 Legend 행
순서를 컬럼 순서에 맞춰 조정. 값/서식 변경 없음.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RLKe4KQFpEQ36hSkMfpEtx
</commit_message>
<xml_diff>
--- a/Content/Data/items/items.xlsx
+++ b/Content/Data/items/items.xlsx
@@ -388,11 +388,11 @@
     <col width="16" customWidth="1" style="7" min="3" max="4"/>
     <col width="12" customWidth="1" style="7" min="5" max="5"/>
     <col width="44" customWidth="1" style="7" min="6" max="6"/>
-    <col width="84.29000000000001" customWidth="1" style="7" min="7" max="7"/>
-    <col width="13" customWidth="1" style="7" min="8" max="8"/>
-    <col width="24" customWidth="1" style="7" min="9" max="11"/>
-    <col width="26" customWidth="1" style="7" min="12" max="14"/>
-    <col width="44" customWidth="1" style="7" min="15" max="15"/>
+    <col width="44" customWidth="1" style="7" min="7" max="7"/>
+    <col width="84.29000000000001" customWidth="1" style="7" min="8" max="8"/>
+    <col width="13" customWidth="1" style="7" min="9" max="9"/>
+    <col width="24" customWidth="1" style="7" min="10" max="12"/>
+    <col width="26" customWidth="1" style="7" min="13" max="15"/>
     <col width="8.710000000000001" customWidth="1" style="7" min="16" max="26"/>
   </cols>
   <sheetData>
@@ -429,47 +429,47 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>HudIconPath</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>ActorClassPath</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>EquipTime</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>PrimarySkillCooldown</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>PrimarySkillManaCost</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>PrimarySkillCastTime</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>SecondarySkillCooldown</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>SecondarySkillManaCost</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>SecondarySkillCastTime</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>HudIconPath</t>
         </is>
       </c>
     </row>
@@ -511,42 +511,42 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
           <t>float</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>float</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>string</t>
         </is>
       </c>
     </row>
@@ -581,17 +581,15 @@
           <t>/Game/UI/Icons/T_Icon_P_1.T_Icon_P_1</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>/Game/Weapons/WK-11_Viper/BP_WK-11_Viper.BP_WK-11_Viper_C</t>
         </is>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="I3" s="6" t="n">
         <v>2.03</v>
       </c>
-      <c r="I3" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="J3" s="6" t="n">
         <v>0</v>
       </c>
@@ -607,7 +605,9 @@
       <c r="N3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O3" s="6" t="n"/>
+      <c r="O3" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -640,17 +640,15 @@
           <t>/Game/UI/Icons/T_Icon_AR_1.T_Icon_AR_1</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>/Game/Weapons/AK105/BP_AK105.BP_AK105_C</t>
         </is>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="I4" s="6" t="n">
         <v>1.55</v>
       </c>
-      <c r="I4" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="J4" s="6" t="n">
         <v>0</v>
       </c>
@@ -666,7 +664,9 @@
       <c r="N4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O4" s="6" t="n"/>
+      <c r="O4" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -699,17 +699,15 @@
           <t>/Game/UI/Icons/T_Icon_AR_2.T_Icon_AR_2</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>/Game/Weapons/TR15/BP_TR15.BP_TR15_C</t>
         </is>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="I5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I5" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="J5" s="6" t="n">
         <v>0</v>
       </c>
@@ -725,7 +723,9 @@
       <c r="N5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O5" s="6" t="n"/>
+      <c r="O5" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -758,17 +758,15 @@
           <t>/Game/UI/Icons/T_Icon_SR_1.T_Icon_SR_1</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>/Game/Weapons/SRM-12/BP_SRM-12.BP_SRM-12_C</t>
         </is>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="I6" s="6" t="n">
         <v>1.8</v>
       </c>
-      <c r="I6" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="J6" s="6" t="n">
         <v>0</v>
       </c>
@@ -784,7 +782,9 @@
       <c r="N6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="6" t="n"/>
+      <c r="O6" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -817,17 +817,15 @@
           <t>/Game/UI/Icons/T_Icon_SMG_1.T_Icon_SMG_1</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>/Game/Weapons/MKR9/BP_MKR9.BP_MKR9_C</t>
         </is>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="I7" s="6" t="n">
         <v>1.13</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="J7" s="6" t="n">
         <v>0</v>
       </c>
@@ -843,7 +841,9 @@
       <c r="N7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O7" s="6" t="n"/>
+      <c r="O7" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -876,17 +876,15 @@
           <t>/Game/UI/Icons/T_Icon_SG_1.T_Icon_SG_1</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>/Game/Weapons/Herrington_11-87/BP_Herrington_11-87_Police.BP_Herrington_11-87_Police_C</t>
         </is>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="I8" s="6" t="n">
         <v>1.8</v>
       </c>
-      <c r="I8" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="J8" s="6" t="n">
         <v>0</v>
       </c>
@@ -902,7 +900,9 @@
       <c r="N8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O8" s="6" t="n"/>
+      <c r="O8" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -935,17 +935,15 @@
           <t>/Game/UI/Icons/T_Icon_SR_2.T_Icon_SR_2</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>/Game/Weapons/MK14EBR/BP_MK14EBR.BP_MK14EBR_C</t>
         </is>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="I9" s="6" t="n">
         <v>1.8</v>
       </c>
-      <c r="I9" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="J9" s="6" t="n">
         <v>0</v>
       </c>
@@ -961,7 +959,9 @@
       <c r="N9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O9" s="6" t="n"/>
+      <c r="O9" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -994,17 +994,15 @@
           <t>/Game/UI/Icons/T_Icon_SMG_2.T_Icon_SMG_2</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>/Game/Weapons/MKR9/BP_MKR9.BP_MKR9_C</t>
         </is>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="I10" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="I10" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="J10" s="6" t="n">
         <v>0</v>
       </c>
@@ -1020,7 +1018,9 @@
       <c r="N10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O10" s="6" t="n"/>
+      <c r="O10" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1053,17 +1053,15 @@
           <t>/Game/UI/Icons/T_Icon_AR_3.T_Icon_AR_3</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>/Game/Weapons/MX68/BP_MX68.BP_MX68_C</t>
         </is>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="I11" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I11" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="J11" s="6" t="n">
         <v>0</v>
       </c>
@@ -1079,7 +1077,9 @@
       <c r="N11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O11" s="6" t="n"/>
+      <c r="O11" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -1112,17 +1112,15 @@
           <t>/Game/UI/Icons/T_Icon_P_2.T_Icon_P_2</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>/Game/Weapons/R08/BP_R08.BP_R08_C</t>
         </is>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="I12" s="6" t="n">
         <v>2.11</v>
       </c>
-      <c r="I12" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="J12" s="6" t="n">
         <v>0</v>
       </c>
@@ -1138,7 +1136,9 @@
       <c r="N12" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O12" s="6" t="n"/>
+      <c r="O12" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="7"/>
     <row r="22" ht="15.75" customHeight="1" s="7"/>
@@ -2140,11 +2140,11 @@
     <col width="16" customWidth="1" style="7" min="3" max="4"/>
     <col width="12" customWidth="1" style="7" min="5" max="5"/>
     <col width="44" customWidth="1" style="7" min="6" max="6"/>
-    <col width="60" customWidth="1" style="7" min="7" max="7"/>
-    <col width="13" customWidth="1" style="7" min="8" max="8"/>
-    <col width="24" customWidth="1" style="7" min="9" max="11"/>
-    <col width="26" customWidth="1" style="7" min="12" max="14"/>
-    <col width="44" customWidth="1" style="7" min="15" max="15"/>
+    <col width="44" customWidth="1" style="7" min="7" max="7"/>
+    <col width="60" customWidth="1" style="7" min="8" max="8"/>
+    <col width="13" customWidth="1" style="7" min="9" max="9"/>
+    <col width="24" customWidth="1" style="7" min="10" max="12"/>
+    <col width="26" customWidth="1" style="7" min="13" max="15"/>
     <col width="8.710000000000001" customWidth="1" style="7" min="16" max="26"/>
   </cols>
   <sheetData>
@@ -2181,47 +2181,47 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>HudIconPath</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>ActorClassPath</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>EquipTime</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>PrimarySkillCooldown</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>PrimarySkillManaCost</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>PrimarySkillCastTime</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>SecondarySkillCooldown</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>SecondarySkillManaCost</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>SecondarySkillCastTime</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>HudIconPath</t>
         </is>
       </c>
     </row>
@@ -2263,42 +2263,42 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
           <t>float</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>float</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>string</t>
         </is>
       </c>
     </row>
@@ -2329,17 +2329,15 @@
         </is>
       </c>
       <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>/Game/Items/Unarmed/BP_Unarmed.BP_Unarmed_C</t>
         </is>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="I3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="J3" s="6" t="n">
         <v>0</v>
       </c>
@@ -2355,7 +2353,9 @@
       <c r="N3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O3" s="6" t="n"/>
+      <c r="O3" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2388,33 +2388,33 @@
           <t>/Game/UI/Icons/T_Icon_I_1.T_Icon_I_1</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>/Game/Items/I_1/BP_I_1.BP_I_1_C</t>
         </is>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="I4" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="J4" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="6" t="n">
+      <c r="K4" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="K4" s="6" t="n">
+      <c r="L4" s="6" t="n">
         <v>0.7</v>
       </c>
-      <c r="L4" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="M4" s="6" t="n">
         <v>0</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O4" s="6" t="n"/>
+      <c r="O4" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2447,33 +2447,33 @@
           <t>/Game/UI/Icons/T_Icon_I_2.T_Icon_I_2</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>/Game/Items/I_2/BP_I_2.BP_I_2_C</t>
         </is>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="I5" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="J5" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="K5" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="L5" s="6" t="n">
         <v>1.2</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="M5" s="6" t="n">
         <v>0</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O5" s="6" t="n"/>
+      <c r="O5" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="7"/>
     <row r="22" ht="15.75" customHeight="1" s="7"/>
@@ -5087,7 +5087,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>ActorClassPath</t>
+          <t>HudIconPath</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -5102,19 +5102,19 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>장착 시 스폰할 Actor 클래스 경로.</t>
+          <t>HUD(우측 하단) 표시용 2D 아이콘 애셋 경로. 없으면 빈 값이며, 이 경우 IconPath를 대신 사용.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>EquipTime</t>
+          <t>ActorClassPath</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -5124,14 +5124,14 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>장착(Draw) 애니메이션 재생 시간(초). weapons.json엔 더 이상 없음.</t>
+          <t>장착 시 스폰할 Actor 클래스 경로.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>PrimarySkillCooldown</t>
+          <t>EquipTime</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -5146,14 +5146,14 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>1번 스킬 쿨다운(초). 없으면 0.</t>
+          <t>장착(Draw) 애니메이션 재생 시간(초). weapons.json엔 더 이상 없음.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>PrimarySkillManaCost</t>
+          <t>PrimarySkillCooldown</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -5168,14 +5168,14 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>1번 스킬 마나 소모량. 없으면 0.</t>
+          <t>1번 스킬 쿨다운(초). 없으면 0.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>PrimarySkillCastTime</t>
+          <t>PrimarySkillManaCost</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -5190,14 +5190,14 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>1번 스킬 시전(Use) 애니메이션 재생 시간(초). 재생 중엔 재발동 불가.</t>
+          <t>1번 스킬 마나 소모량. 없으면 0.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>SecondarySkillCooldown</t>
+          <t>PrimarySkillCastTime</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -5212,14 +5212,14 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>2번 스킬 쿨다운(초). 없으면 0.</t>
+          <t>1번 스킬 시전(Use) 애니메이션 재생 시간(초). 재생 중엔 재발동 불가.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>SecondarySkillManaCost</t>
+          <t>SecondarySkillCooldown</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -5234,14 +5234,14 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>2번 스킬 마나 소모량. 없으면 0.</t>
+          <t>2번 스킬 쿨다운(초). 없으면 0.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>SecondarySkillCastTime</t>
+          <t>SecondarySkillManaCost</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -5256,19 +5256,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>2번 스킬 시전(Use) 애니메이션 재생 시간(초).</t>
+          <t>2번 스킬 마나 소모량. 없으면 0.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>HudIconPath</t>
+          <t>SecondarySkillCastTime</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>float</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>HUD(우측 하단) 표시용 2D 아이콘 애셋 경로. 없으면 빈 값이며, 이 경우 IconPath를 대신 사용.</t>
+          <t>2번 스킬 시전(Use) 애니메이션 재생 시간(초).</t>
         </is>
       </c>
     </row>

</xml_diff>